<commit_message>
removed timezone adjustment to accomadate beijing time
</commit_message>
<xml_diff>
--- a/data/cleaned_gas_prices.xlsx
+++ b/data/cleaned_gas_prices.xlsx
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>45887.2341087963</v>
+        <v>45887.8591087963</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -529,7 +529,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K2" s="2" t="n">
@@ -556,7 +556,7 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>45887.2341087963</v>
+        <v>45887.8591087963</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -576,7 +576,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K3" s="2" t="n">
@@ -603,7 +603,7 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>45887.23504629629</v>
+        <v>45887.86004629629</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -623,7 +623,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K4" s="2" t="n">
@@ -650,7 +650,7 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>45887.23504629629</v>
+        <v>45887.86004629629</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -670,7 +670,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K5" s="2" t="n">
@@ -697,7 +697,7 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>45887.23592592592</v>
+        <v>45887.86092592592</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -717,7 +717,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K6" s="2" t="n">
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>45887.23592592592</v>
+        <v>45887.86092592592</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -764,7 +764,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K7" s="2" t="n">
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>45887.2341087963</v>
+        <v>45887.8591087963</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -811,7 +811,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K8" s="2" t="n">
@@ -838,7 +838,7 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>45887.2341087963</v>
+        <v>45887.8591087963</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -858,7 +858,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K9" s="2" t="n">
@@ -885,7 +885,7 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>45887.2341087963</v>
+        <v>45887.8591087963</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -905,7 +905,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K10" s="2" t="n">
@@ -932,7 +932,7 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>45887.2341087963</v>
+        <v>45887.8591087963</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -952,7 +952,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K11" s="2" t="n">
@@ -979,7 +979,7 @@
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>45887.2341087963</v>
+        <v>45887.8591087963</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -999,7 +999,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K12" s="2" t="n">
@@ -1026,7 +1026,7 @@
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>45887.23504629629</v>
+        <v>45887.86004629629</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -1046,7 +1046,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K13" s="2" t="n">
@@ -1073,7 +1073,7 @@
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>45887.23504629629</v>
+        <v>45887.86004629629</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -1093,7 +1093,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K14" s="2" t="n">
@@ -1120,7 +1120,7 @@
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>45887.2341087963</v>
+        <v>45887.8591087963</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -1140,7 +1140,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K15" s="2" t="n">
@@ -1167,7 +1167,7 @@
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>45887.23504629629</v>
+        <v>45887.86004629629</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -1187,7 +1187,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K16" s="2" t="n">
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>45887.2341087963</v>
+        <v>45887.8591087963</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -1234,7 +1234,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K17" s="2" t="n">
@@ -1261,7 +1261,7 @@
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>45887.2341087963</v>
+        <v>45887.8591087963</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K18" s="2" t="n">
@@ -1308,7 +1308,7 @@
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>45887.2341087963</v>
+        <v>45887.8591087963</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1328,7 +1328,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K19" s="2" t="n">
@@ -1355,7 +1355,7 @@
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>45887.2341087963</v>
+        <v>45887.8591087963</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K20" s="2" t="n">
@@ -1402,7 +1402,7 @@
         </is>
       </c>
       <c r="E21" s="2" t="n">
-        <v>45887.23592592592</v>
+        <v>45887.86092592592</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1422,7 +1422,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K21" s="2" t="n">
@@ -1449,7 +1449,7 @@
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>45887.2341087963</v>
+        <v>45887.8591087963</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -1469,7 +1469,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K22" s="2" t="n">
@@ -1496,7 +1496,7 @@
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>45887.23592592592</v>
+        <v>45887.86092592592</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -1516,7 +1516,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K23" s="2" t="n">
@@ -1543,7 +1543,7 @@
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>45887.2341087963</v>
+        <v>45887.8591087963</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1563,7 +1563,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K24" s="2" t="n">
@@ -1590,7 +1590,7 @@
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>45887.23504629629</v>
+        <v>45887.86004629629</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -1610,7 +1610,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K25" s="2" t="n">
@@ -1637,7 +1637,7 @@
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>45887.23504629629</v>
+        <v>45887.86004629629</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -1657,7 +1657,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K26" s="2" t="n">
@@ -1684,7 +1684,7 @@
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>45887.23504629629</v>
+        <v>45887.86004629629</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -1704,7 +1704,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K27" s="2" t="n">
@@ -1731,7 +1731,7 @@
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>45887.23504629629</v>
+        <v>45887.86004629629</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1751,7 +1751,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K28" s="2" t="n">
@@ -1778,7 +1778,7 @@
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>45887.23504629629</v>
+        <v>45887.86004629629</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K29" s="2" t="n">
@@ -1825,7 +1825,7 @@
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>45887.23592592592</v>
+        <v>45887.86092592592</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -1845,7 +1845,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K30" s="2" t="n">
@@ -1872,7 +1872,7 @@
         </is>
       </c>
       <c r="E31" s="2" t="n">
-        <v>45887.23504629629</v>
+        <v>45887.86004629629</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -1892,7 +1892,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K31" s="2" t="n">
@@ -1919,7 +1919,7 @@
         </is>
       </c>
       <c r="E32" s="2" t="n">
-        <v>45887.23504629629</v>
+        <v>45887.86004629629</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -1939,7 +1939,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K32" s="2" t="n">
@@ -1966,7 +1966,7 @@
         </is>
       </c>
       <c r="E33" s="2" t="n">
-        <v>45887.2341087963</v>
+        <v>45887.8591087963</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -1986,7 +1986,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K33" s="2" t="n">
@@ -2013,7 +2013,7 @@
         </is>
       </c>
       <c r="E34" s="2" t="n">
-        <v>45887.23504629629</v>
+        <v>45887.86004629629</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -2033,7 +2033,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K34" s="2" t="n">
@@ -2060,7 +2060,7 @@
         </is>
       </c>
       <c r="E35" s="2" t="n">
-        <v>45887.23504629629</v>
+        <v>45887.86004629629</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -2080,7 +2080,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K35" s="2" t="n">
@@ -2107,7 +2107,7 @@
         </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>45887.23504629629</v>
+        <v>45887.86004629629</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -2127,7 +2127,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K36" s="2" t="n">
@@ -2154,7 +2154,7 @@
         </is>
       </c>
       <c r="E37" s="2" t="n">
-        <v>45887.2341087963</v>
+        <v>45887.8591087963</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -2174,7 +2174,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K37" s="2" t="n">
@@ -2201,7 +2201,7 @@
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>45887.23504629629</v>
+        <v>45887.86004629629</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -2221,7 +2221,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K38" s="2" t="n">
@@ -2248,7 +2248,7 @@
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>45887.2341087963</v>
+        <v>45887.8591087963</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -2268,7 +2268,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K39" s="2" t="n">
@@ -2295,7 +2295,7 @@
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>45887.23504629629</v>
+        <v>45887.86004629629</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
@@ -2315,7 +2315,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K40" s="2" t="n">
@@ -2342,7 +2342,7 @@
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>45887.2341087963</v>
+        <v>45887.8591087963</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
@@ -2362,7 +2362,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K41" s="2" t="n">
@@ -2389,7 +2389,7 @@
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>45887.2341087963</v>
+        <v>45887.8591087963</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
@@ -2409,7 +2409,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K42" s="2" t="n">
@@ -2436,7 +2436,7 @@
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>45887.2341087963</v>
+        <v>45887.8591087963</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
@@ -2456,7 +2456,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K43" s="2" t="n">
@@ -2483,7 +2483,7 @@
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>45887.23592592592</v>
+        <v>45887.86092592592</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
@@ -2494,14 +2494,14 @@
         <v>167.9</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>45887.23592592592</v>
+        <v>45887.86092592592</v>
       </c>
       <c r="I44" t="n">
         <v>0</v>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K44" s="2" t="n">
@@ -2528,7 +2528,7 @@
         </is>
       </c>
       <c r="E45" s="2" t="n">
-        <v>45887.23504629629</v>
+        <v>45887.86004629629</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
@@ -2548,7 +2548,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>midnight</t>
+          <t>evening</t>
         </is>
       </c>
       <c r="K45" s="2" t="n">

</xml_diff>